<commit_message>
[auto] session sync 2026-07-23T00:47:10Z
</commit_message>
<xml_diff>
--- a/2D 자동 제작도 개발 현황.xlsx
+++ b/2D 자동 제작도 개발 현황.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\duddl\Desktop\Project\a2z\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F187E248-2EF2-4954-B040-2A45F3210D00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC6A772-55AC-4F2B-A523-AE28161FEB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="489">
   <si>
     <t>2D 자동 제작도 개발 현황</t>
   </si>
@@ -1048,12 +1048,6 @@
     <t>고정 열 너비 + 폰트 축소</t>
   </si>
   <si>
-    <t>앱/템플릿 조정</t>
-  </si>
-  <si>
-    <t>SPREF 실제 샘플과 표준 약어 결정 필요</t>
-  </si>
-  <si>
     <t>조립도</t>
   </si>
   <si>
@@ -1493,6 +1487,26 @@
   </si>
   <si>
     <t>낮은 우선순위이며 아직 요청 미전달</t>
+  </si>
+  <si>
+    <t>O</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>완료</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>없음</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>X</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>BOM 텍스트 줄바꿈·열 너비 실기 확인 완료</t>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1902,7 +1916,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1933,17 +1947,44 @@
     <xf numFmtId="176" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1987,13 +2028,16 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1">
@@ -2031,42 +2075,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2603,28 +2611,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3"/>
@@ -2635,54 +2643,54 @@
       <c r="F3"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="22" t="s">
+      <c r="B4" s="26"/>
+      <c r="C4" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="24" t="s">
+      <c r="D4" s="32"/>
+      <c r="E4" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="25"/>
-      <c r="G4" s="26" t="s">
+      <c r="F4" s="34"/>
+      <c r="G4" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="27"/>
+      <c r="H4" s="36"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A5" s="18">
+      <c r="A5" s="27">
         <f>COUNTA('개발 항목'!$D$6:$D$79)</f>
         <v>74</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="18">
+      <c r="B5" s="28"/>
+      <c r="C5" s="27">
         <f>COUNTIF('개발 항목'!$I$6:$I$79,"완료")</f>
-        <v>27</v>
-      </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="18">
+        <v>28</v>
+      </c>
+      <c r="D5" s="28"/>
+      <c r="E5" s="27">
         <f>COUNTIF('개발 항목'!$I$6:$I$79,"실기 검증 대기")</f>
         <v>10</v>
       </c>
-      <c r="F5" s="19"/>
-      <c r="G5" s="18">
+      <c r="F5" s="28"/>
+      <c r="G5" s="27">
         <f>COUNTIFS('개발 항목'!$E$6:$E$79,"○",'개발 항목'!$H$6:$H$79,"&lt;&gt;O")</f>
         <v>35</v>
       </c>
-      <c r="H5" s="19"/>
+      <c r="H5" s="28"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A6" s="20"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="21"/>
+      <c r="A6" s="29"/>
+      <c r="B6" s="30"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="30"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A7"/>
@@ -2693,16 +2701,16 @@
       <c r="F7"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="6" t="s">
@@ -2973,89 +2981,96 @@
       <c r="F19"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
+      <c r="B20" s="40"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="40"/>
+      <c r="E20" s="40"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="40"/>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="12"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="38"/>
+      <c r="H21" s="39"/>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="37" t="s">
         <v>205</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="12"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="39"/>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="12"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="39"/>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="37" t="s">
         <v>206</v>
       </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="12"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="39"/>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="12"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B21:H21"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:B4"/>
@@ -3066,13 +3081,6 @@
     <mergeCell ref="E5:F6"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="G5:H6"/>
-    <mergeCell ref="B24:H24"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="B21:H21"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3092,7 +3100,7 @@
     <col min="6" max="6" width="13.19921875" style="5" customWidth="1"/>
     <col min="7" max="7" width="15" style="5" customWidth="1"/>
     <col min="8" max="8" width="15.5" customWidth="1"/>
-    <col min="9" max="9" width="15.5" style="53" customWidth="1"/>
+    <col min="9" max="9" width="15.5" style="16" customWidth="1"/>
     <col min="10" max="10" width="37" style="5" customWidth="1"/>
     <col min="11" max="11" width="17.19921875" style="5" customWidth="1"/>
     <col min="12" max="13" width="13.69921875" customWidth="1"/>
@@ -3103,70 +3111,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
-      <c r="Q1" s="28"/>
-      <c r="R1" s="28"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.4">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-      <c r="P2" s="29"/>
-      <c r="Q2" s="29"/>
-      <c r="R2" s="29"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.4">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="30"/>
-      <c r="O3" s="30"/>
-      <c r="P3" s="30"/>
-      <c r="Q3" s="30"/>
-      <c r="R3" s="30"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
     </row>
     <row r="5" spans="1:18" ht="43.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="6" t="s">
@@ -3233,7 +3241,7 @@
         <v>207</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="E6" s="8" t="s">
         <v>76</v>
@@ -3251,10 +3259,10 @@
         <v>162</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="L6" s="8" t="s">
         <v>54</v>
@@ -3270,7 +3278,7 @@
         <v>46225</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="R6"/>
     </row>
@@ -3279,13 +3287,13 @@
         <v>51</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>292</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>55</v>
@@ -3300,10 +3308,10 @@
         <v>246</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="K7" s="8" t="s">
         <v>79</v>
@@ -3322,7 +3330,7 @@
         <v>46226</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="R7"/>
     </row>
@@ -3547,13 +3555,13 @@
         <v>15</v>
       </c>
       <c r="B12" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>339</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>340</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>341</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>76</v>
@@ -3571,7 +3579,7 @@
         <v>2</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="K12" s="8" t="s">
         <v>79</v>
@@ -3592,7 +3600,7 @@
         <v>46225</v>
       </c>
       <c r="Q12" s="7" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="R12"/>
     </row>
@@ -3601,13 +3609,13 @@
         <v>16</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>76</v>
@@ -3625,7 +3633,7 @@
         <v>2</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="K13" s="8" t="s">
         <v>79</v>
@@ -3646,7 +3654,7 @@
         <v>46225</v>
       </c>
       <c r="Q13" s="7" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="R13"/>
     </row>
@@ -3661,7 +3669,7 @@
         <v>249</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>76</v>
@@ -3679,7 +3687,7 @@
         <v>2</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="K14" s="8" t="s">
         <v>79</v>
@@ -3698,7 +3706,7 @@
         <v>46224</v>
       </c>
       <c r="Q14" s="7" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="R14"/>
     </row>
@@ -3713,7 +3721,7 @@
         <v>190</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>113</v>
@@ -3731,7 +3739,7 @@
         <v>2</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="K15" s="8" t="s">
         <v>79</v>
@@ -3750,7 +3758,7 @@
         <v>46156</v>
       </c>
       <c r="Q15" s="7" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="R15"/>
     </row>
@@ -3762,7 +3770,7 @@
         <v>212</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>141</v>
@@ -3783,7 +3791,7 @@
         <v>2</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="K16" s="8" t="s">
         <v>79</v>
@@ -3804,7 +3812,7 @@
         <v>46224</v>
       </c>
       <c r="Q16" s="7" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="R16"/>
     </row>
@@ -3816,10 +3824,10 @@
         <v>212</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>55</v>
@@ -3837,7 +3845,7 @@
         <v>2</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="K17" s="8" t="s">
         <v>79</v>
@@ -3858,7 +3866,7 @@
         <v>46225</v>
       </c>
       <c r="Q17" s="7" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="R17"/>
     </row>
@@ -3870,10 +3878,10 @@
         <v>212</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>55</v>
@@ -3891,7 +3899,7 @@
         <v>2</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="K18" s="8" t="s">
         <v>79</v>
@@ -3910,7 +3918,7 @@
         <v>46223</v>
       </c>
       <c r="Q18" s="7" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="R18"/>
     </row>
@@ -3925,7 +3933,7 @@
         <v>249</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>76</v>
@@ -3943,7 +3951,7 @@
         <v>2</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="K19" s="8" t="s">
         <v>79</v>
@@ -3962,7 +3970,7 @@
         <v>46156</v>
       </c>
       <c r="Q19" s="7" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="R19"/>
     </row>
@@ -3977,7 +3985,7 @@
         <v>249</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="E20" s="8" t="s">
         <v>76</v>
@@ -3995,7 +4003,7 @@
         <v>2</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="K20" s="8" t="s">
         <v>79</v>
@@ -4014,7 +4022,7 @@
         <v>46156</v>
       </c>
       <c r="Q20" s="7" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="R20"/>
     </row>
@@ -4029,7 +4037,7 @@
         <v>249</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>76</v>
@@ -4047,7 +4055,7 @@
         <v>2</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="K21" s="8" t="s">
         <v>79</v>
@@ -4066,7 +4074,7 @@
         <v>46156</v>
       </c>
       <c r="Q21" s="7" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="R21"/>
     </row>
@@ -4078,10 +4086,10 @@
         <v>240</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>76</v>
@@ -4099,7 +4107,7 @@
         <v>2</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="K22" s="8" t="s">
         <v>79</v>
@@ -4118,7 +4126,7 @@
         <v>46156</v>
       </c>
       <c r="Q22" s="7" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="R22"/>
     </row>
@@ -4133,7 +4141,7 @@
         <v>185</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>76</v>
@@ -4151,7 +4159,7 @@
         <v>2</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="K23" s="8" t="s">
         <v>79</v>
@@ -4170,7 +4178,7 @@
         <v>46225</v>
       </c>
       <c r="Q23" s="7" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="R23"/>
     </row>
@@ -4203,7 +4211,7 @@
         <v>2</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="K24" s="8" t="s">
         <v>79</v>
@@ -4222,7 +4230,7 @@
         <v>46156</v>
       </c>
       <c r="Q24" s="7" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="R24"/>
     </row>
@@ -4237,7 +4245,7 @@
         <v>185</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>76</v>
@@ -4255,7 +4263,7 @@
         <v>2</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="K25" s="8" t="s">
         <v>79</v>
@@ -4276,7 +4284,7 @@
         <v>46226</v>
       </c>
       <c r="Q25" s="7" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="R25"/>
     </row>
@@ -4309,7 +4317,7 @@
         <v>2</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="K26" s="8" t="s">
         <v>79</v>
@@ -4361,7 +4369,7 @@
         <v>2</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="K27" s="8" t="s">
         <v>79</v>
@@ -4380,7 +4388,7 @@
         <v>46224</v>
       </c>
       <c r="Q27" s="7" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="R27"/>
     </row>
@@ -4389,13 +4397,13 @@
         <v>31</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>185</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="E28" s="8" t="s">
         <v>76</v>
@@ -4413,7 +4421,7 @@
         <v>2</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="K28" s="8" t="s">
         <v>79</v>
@@ -4434,7 +4442,7 @@
         <v>46225</v>
       </c>
       <c r="Q28" s="7" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="R28"/>
     </row>
@@ -4443,13 +4451,13 @@
         <v>49</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>292</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E29" s="8" t="s">
         <v>76</v>
@@ -4467,7 +4475,7 @@
         <v>2</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="K29" s="8" t="s">
         <v>79</v>
@@ -4488,7 +4496,7 @@
         <v>46224</v>
       </c>
       <c r="Q29" s="7" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="R29"/>
     </row>
@@ -4503,7 +4511,7 @@
         <v>292</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>76</v>
@@ -4521,7 +4529,7 @@
         <v>2</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="K30" s="8" t="s">
         <v>79</v>
@@ -4542,7 +4550,7 @@
         <v>46224</v>
       </c>
       <c r="Q30" s="7" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="R30"/>
     </row>
@@ -4554,10 +4562,10 @@
         <v>171</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E31" s="8" t="s">
         <v>55</v>
@@ -4575,7 +4583,7 @@
         <v>2</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="K31" s="8" t="s">
         <v>79</v>
@@ -4596,7 +4604,7 @@
         <v>46222</v>
       </c>
       <c r="Q31" s="7" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="R31"/>
     </row>
@@ -4608,10 +4616,10 @@
         <v>171</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E32" s="8" t="s">
         <v>55</v>
@@ -4629,7 +4637,7 @@
         <v>2</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="K32" s="8" t="s">
         <v>79</v>
@@ -4650,7 +4658,7 @@
         <v>46225</v>
       </c>
       <c r="Q32" s="7" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="R32"/>
     </row>
@@ -4662,10 +4670,10 @@
         <v>240</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="E33" s="8" t="s">
         <v>55</v>
@@ -4683,7 +4691,7 @@
         <v>2</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="K33" s="8" t="s">
         <v>79</v>
@@ -4704,61 +4712,61 @@
         <v>46225</v>
       </c>
       <c r="Q33" s="7" t="s">
+        <v>453</v>
+      </c>
+      <c r="R33"/>
+    </row>
+    <row r="34" spans="1:18" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="10">
+        <v>69</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>454</v>
+      </c>
+      <c r="D34" s="10" t="s">
         <v>455</v>
       </c>
-      <c r="R33"/>
-    </row>
-    <row r="34" spans="1:18" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="43">
-        <v>69</v>
-      </c>
-      <c r="B34" s="43" t="s">
-        <v>240</v>
-      </c>
-      <c r="C34" s="43" t="s">
+      <c r="E34" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G34" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I34" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="J34" s="10" t="s">
         <v>456</v>
       </c>
-      <c r="D34" s="43" t="s">
+      <c r="K34" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="L34" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="M34" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="N34" s="13">
+        <v>46225</v>
+      </c>
+      <c r="O34" s="13">
+        <v>46225</v>
+      </c>
+      <c r="P34" s="13">
+        <v>46225</v>
+      </c>
+      <c r="Q34" s="10" t="s">
         <v>457</v>
-      </c>
-      <c r="E34" s="43" t="s">
-        <v>76</v>
-      </c>
-      <c r="F34" s="43" t="s">
-        <v>55</v>
-      </c>
-      <c r="G34" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="H34" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="I34" s="43" t="s">
-        <v>2</v>
-      </c>
-      <c r="J34" s="43" t="s">
-        <v>458</v>
-      </c>
-      <c r="K34" s="43" t="s">
-        <v>79</v>
-      </c>
-      <c r="L34" s="43" t="s">
-        <v>55</v>
-      </c>
-      <c r="M34" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="N34" s="46">
-        <v>46225</v>
-      </c>
-      <c r="O34" s="46">
-        <v>46225</v>
-      </c>
-      <c r="P34" s="46">
-        <v>46225</v>
-      </c>
-      <c r="Q34" s="43" t="s">
-        <v>459</v>
       </c>
       <c r="R34"/>
     </row>
@@ -4926,10 +4934,10 @@
         <v>166</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E38" s="8" t="s">
         <v>76</v>
@@ -4947,7 +4955,7 @@
         <v>3</v>
       </c>
       <c r="J38" s="7" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="K38" s="8" t="s">
         <v>79</v>
@@ -4966,7 +4974,7 @@
         <v>46224</v>
       </c>
       <c r="Q38" s="7" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="R38"/>
     </row>
@@ -4975,13 +4983,13 @@
         <v>18</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="E39" s="8" t="s">
         <v>76</v>
@@ -4999,7 +5007,7 @@
         <v>3</v>
       </c>
       <c r="J39" s="7" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="K39" s="8" t="s">
         <v>79</v>
@@ -5018,7 +5026,7 @@
         <v>46224</v>
       </c>
       <c r="Q39" s="7" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="R39"/>
     </row>
@@ -5033,7 +5041,7 @@
         <v>292</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="E40" s="8" t="s">
         <v>76</v>
@@ -5051,7 +5059,7 @@
         <v>3</v>
       </c>
       <c r="J40" s="7" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="K40" s="8" t="s">
         <v>79</v>
@@ -5070,7 +5078,7 @@
         <v>46225</v>
       </c>
       <c r="Q40" s="7" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="R40"/>
     </row>
@@ -5085,7 +5093,7 @@
         <v>297</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="E41" s="8" t="s">
         <v>76</v>
@@ -5103,7 +5111,7 @@
         <v>3</v>
       </c>
       <c r="J41" s="7" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="K41" s="8" t="s">
         <v>79</v>
@@ -5122,7 +5130,7 @@
         <v>46225</v>
       </c>
       <c r="Q41" s="7" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="R41"/>
     </row>
@@ -5137,7 +5145,7 @@
         <v>297</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E42" s="8" t="s">
         <v>76</v>
@@ -5155,7 +5163,7 @@
         <v>3</v>
       </c>
       <c r="J42" s="7" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="K42" s="8" t="s">
         <v>79</v>
@@ -5174,7 +5182,7 @@
         <v>46225</v>
       </c>
       <c r="Q42" s="7" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="R42"/>
     </row>
@@ -5186,10 +5194,10 @@
         <v>160</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E43" s="8" t="s">
         <v>76</v>
@@ -5207,7 +5215,7 @@
         <v>3</v>
       </c>
       <c r="J43" s="7" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="K43" s="8" t="s">
         <v>304</v>
@@ -5226,7 +5234,7 @@
         <v>46225</v>
       </c>
       <c r="Q43" s="7" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="R43"/>
     </row>
@@ -5238,10 +5246,10 @@
         <v>160</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="E44" s="8" t="s">
         <v>55</v>
@@ -5259,7 +5267,7 @@
         <v>3</v>
       </c>
       <c r="J44" s="7" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="K44" s="8" t="s">
         <v>79</v>
@@ -5278,7 +5286,7 @@
         <v>46225</v>
       </c>
       <c r="Q44" s="7" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="R44"/>
     </row>
@@ -5443,7 +5451,7 @@
         <v>190</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="E48" s="8" t="s">
         <v>113</v>
@@ -5478,7 +5486,7 @@
         <v>46225</v>
       </c>
       <c r="Q48" s="7" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="R48"/>
     </row>
@@ -5490,10 +5498,10 @@
         <v>171</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="E49" s="8" t="s">
         <v>55</v>
@@ -5511,10 +5519,10 @@
         <v>114</v>
       </c>
       <c r="J49" s="7" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="K49" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="L49" s="8" t="s">
         <v>54</v>
@@ -5530,7 +5538,7 @@
         <v>46225</v>
       </c>
       <c r="Q49" s="7" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="R49"/>
     </row>
@@ -5542,10 +5550,10 @@
         <v>160</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E50" s="8" t="s">
         <v>55</v>
@@ -5563,7 +5571,7 @@
         <v>114</v>
       </c>
       <c r="J50" s="7" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="K50" s="8" t="s">
         <v>210</v>
@@ -5580,7 +5588,7 @@
         <v>46224</v>
       </c>
       <c r="Q50" s="7" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="R50"/>
     </row>
@@ -6022,22 +6030,22 @@
         <v>76</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>113</v>
+        <v>484</v>
       </c>
       <c r="H59" s="8" t="s">
-        <v>273</v>
+        <v>484</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>85</v>
+        <v>485</v>
       </c>
       <c r="J59" s="7" t="s">
         <v>336</v>
       </c>
       <c r="K59" s="8" t="s">
-        <v>337</v>
+        <v>486</v>
       </c>
       <c r="L59" s="8" t="s">
-        <v>54</v>
+        <v>487</v>
       </c>
       <c r="M59" s="8" t="s">
         <v>55</v>
@@ -6045,12 +6053,14 @@
       <c r="N59" s="9">
         <v>46152</v>
       </c>
-      <c r="O59" s="9"/>
+      <c r="O59" s="9">
+        <v>46226</v>
+      </c>
       <c r="P59" s="9">
-        <v>46155</v>
+        <v>46226</v>
       </c>
       <c r="Q59" s="7" t="s">
-        <v>338</v>
+        <v>488</v>
       </c>
       <c r="R59"/>
     </row>
@@ -6062,10 +6072,10 @@
         <v>240</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="E60" s="8" t="s">
         <v>55</v>
@@ -6083,10 +6093,10 @@
         <v>85</v>
       </c>
       <c r="J60" s="7" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="K60" s="8" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="L60" s="8" t="s">
         <v>54</v>
@@ -6102,7 +6112,7 @@
         <v>46225</v>
       </c>
       <c r="Q60" s="7" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="R60"/>
     </row>
@@ -6674,10 +6684,10 @@
         <v>220</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D72" s="7" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E72" s="8" t="s">
         <v>55</v>
@@ -6692,13 +6702,13 @@
         <v>246</v>
       </c>
       <c r="I72" s="8" t="s">
+        <v>405</v>
+      </c>
+      <c r="J72" s="7" t="s">
+        <v>406</v>
+      </c>
+      <c r="K72" s="8" t="s">
         <v>407</v>
-      </c>
-      <c r="J72" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="K72" s="8" t="s">
-        <v>409</v>
       </c>
       <c r="L72" s="8" t="s">
         <v>55</v>
@@ -6712,7 +6722,7 @@
         <v>46225</v>
       </c>
       <c r="Q72" s="7" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="R72"/>
     </row>
@@ -6921,152 +6931,152 @@
       </c>
     </row>
     <row r="77" spans="1:18" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A77" s="44">
+      <c r="A77" s="11">
         <v>32</v>
       </c>
-      <c r="B77" s="44" t="s">
+      <c r="B77" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="C77" s="44" t="s">
+      <c r="C77" s="11" t="s">
         <v>330</v>
       </c>
-      <c r="D77" s="45" t="s">
+      <c r="D77" s="12" t="s">
         <v>331</v>
       </c>
-      <c r="E77" s="44" t="s">
-        <v>55</v>
-      </c>
-      <c r="F77" s="44" t="s">
-        <v>76</v>
-      </c>
-      <c r="G77" s="44" t="s">
+      <c r="E77" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F77" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="G77" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="H77" s="44" t="s">
-        <v>55</v>
-      </c>
-      <c r="I77" s="44" t="s">
+      <c r="H77" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="I77" s="11" t="s">
         <v>173</v>
       </c>
-      <c r="J77" s="45" t="s">
+      <c r="J77" s="12" t="s">
         <v>332</v>
       </c>
-      <c r="K77" s="44" t="s">
+      <c r="K77" s="11" t="s">
         <v>252</v>
       </c>
-      <c r="L77" s="44" t="s">
-        <v>54</v>
-      </c>
-      <c r="M77" s="44" t="s">
-        <v>54</v>
-      </c>
-      <c r="N77" s="47">
+      <c r="L77" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="M77" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="N77" s="14">
         <v>46224</v>
       </c>
-      <c r="O77" s="47"/>
-      <c r="P77" s="47">
+      <c r="O77" s="14"/>
+      <c r="P77" s="14">
         <v>46225</v>
       </c>
-      <c r="Q77" s="45" t="s">
+      <c r="Q77" s="12" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="78" spans="1:18" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A78" s="48">
+      <c r="A78">
         <v>70</v>
       </c>
-      <c r="B78" s="48" t="s">
+      <c r="B78" t="s">
         <v>212</v>
       </c>
-      <c r="C78" s="48" t="s">
+      <c r="C78" t="s">
         <v>330</v>
       </c>
-      <c r="D78" s="48" t="s">
+      <c r="D78" t="s">
+        <v>458</v>
+      </c>
+      <c r="E78" t="s">
+        <v>76</v>
+      </c>
+      <c r="F78" t="s">
+        <v>55</v>
+      </c>
+      <c r="G78" t="s">
+        <v>55</v>
+      </c>
+      <c r="H78" t="s">
+        <v>55</v>
+      </c>
+      <c r="I78" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="J78" t="s">
+        <v>459</v>
+      </c>
+      <c r="K78" t="s">
+        <v>252</v>
+      </c>
+      <c r="L78" t="s">
+        <v>54</v>
+      </c>
+      <c r="M78" t="s">
+        <v>54</v>
+      </c>
+      <c r="N78" s="15"/>
+      <c r="O78" s="15"/>
+      <c r="P78" s="15">
+        <v>46225</v>
+      </c>
+      <c r="Q78" t="s">
         <v>460</v>
       </c>
-      <c r="E78" s="48" t="s">
-        <v>76</v>
-      </c>
-      <c r="F78" s="48" t="s">
-        <v>55</v>
-      </c>
-      <c r="G78" s="48" t="s">
-        <v>55</v>
-      </c>
-      <c r="H78" s="48" t="s">
-        <v>55</v>
-      </c>
-      <c r="I78" s="54" t="s">
+    </row>
+    <row r="79" spans="1:18" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A79">
+        <v>71</v>
+      </c>
+      <c r="B79" t="s">
+        <v>212</v>
+      </c>
+      <c r="C79" t="s">
+        <v>330</v>
+      </c>
+      <c r="D79" t="s">
+        <v>461</v>
+      </c>
+      <c r="E79" t="s">
+        <v>55</v>
+      </c>
+      <c r="F79" t="s">
+        <v>76</v>
+      </c>
+      <c r="G79" t="s">
+        <v>55</v>
+      </c>
+      <c r="H79" t="s">
+        <v>55</v>
+      </c>
+      <c r="I79" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="J78" s="48" t="s">
-        <v>461</v>
-      </c>
-      <c r="K78" s="48" t="s">
-        <v>252</v>
-      </c>
-      <c r="L78" s="48" t="s">
-        <v>54</v>
-      </c>
-      <c r="M78" s="48" t="s">
-        <v>54</v>
-      </c>
-      <c r="N78" s="49"/>
-      <c r="O78" s="49"/>
-      <c r="P78" s="49">
+      <c r="J79" t="s">
+        <v>462</v>
+      </c>
+      <c r="K79" t="s">
+        <v>257</v>
+      </c>
+      <c r="L79" t="s">
+        <v>55</v>
+      </c>
+      <c r="M79" t="s">
+        <v>54</v>
+      </c>
+      <c r="N79" s="15"/>
+      <c r="O79" s="15"/>
+      <c r="P79" s="15">
         <v>46225</v>
       </c>
-      <c r="Q78" s="48" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="79" spans="1:18" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A79" s="48">
-        <v>71</v>
-      </c>
-      <c r="B79" s="48" t="s">
-        <v>212</v>
-      </c>
-      <c r="C79" s="48" t="s">
-        <v>330</v>
-      </c>
-      <c r="D79" s="48" t="s">
+      <c r="Q79" t="s">
         <v>463</v>
-      </c>
-      <c r="E79" s="48" t="s">
-        <v>55</v>
-      </c>
-      <c r="F79" s="48" t="s">
-        <v>76</v>
-      </c>
-      <c r="G79" s="48" t="s">
-        <v>55</v>
-      </c>
-      <c r="H79" s="48" t="s">
-        <v>55</v>
-      </c>
-      <c r="I79" s="54" t="s">
-        <v>173</v>
-      </c>
-      <c r="J79" s="48" t="s">
-        <v>464</v>
-      </c>
-      <c r="K79" s="48" t="s">
-        <v>257</v>
-      </c>
-      <c r="L79" s="48" t="s">
-        <v>55</v>
-      </c>
-      <c r="M79" s="48" t="s">
-        <v>54</v>
-      </c>
-      <c r="N79" s="49"/>
-      <c r="O79" s="49"/>
-      <c r="P79" s="49">
-        <v>46225</v>
-      </c>
-      <c r="Q79" s="48" t="s">
-        <v>465</v>
       </c>
     </row>
   </sheetData>
@@ -7200,37 +7210,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
     </row>
     <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
+      <c r="B4" s="52"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="52"/>
     </row>
     <row r="5" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
@@ -7348,15 +7358,15 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="52" t="s">
         <v>69</v>
       </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="52"/>
+      <c r="D11" s="52"/>
+      <c r="E11" s="52"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="52"/>
     </row>
     <row r="12" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
@@ -7406,7 +7416,7 @@
     </row>
     <row r="14" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="3" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>76</v>
@@ -7415,16 +7425,16 @@
         <v>2</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>79</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
@@ -7566,15 +7576,15 @@
       </c>
     </row>
     <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="42" t="s">
+      <c r="A22" s="52" t="s">
         <v>105</v>
       </c>
-      <c r="B22" s="42"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="52"/>
+      <c r="D22" s="52"/>
+      <c r="E22" s="52"/>
+      <c r="F22" s="52"/>
+      <c r="G22" s="52"/>
     </row>
     <row r="23" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
@@ -7601,7 +7611,7 @@
     </row>
     <row r="24" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>76</v>
@@ -7610,16 +7620,16 @@
         <v>192</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>94</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
@@ -7853,15 +7863,15 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A36" s="31" t="s">
+      <c r="A36" s="41" t="s">
         <v>148</v>
       </c>
-      <c r="B36" s="31"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="31"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="31"/>
+      <c r="B36" s="41"/>
+      <c r="C36" s="41"/>
+      <c r="D36" s="41"/>
+      <c r="E36" s="41"/>
+      <c r="F36" s="41"/>
+      <c r="G36" s="41"/>
     </row>
     <row r="37" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="6" t="s">
@@ -7911,16 +7921,16 @@
     </row>
     <row r="39" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="7" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B39" s="7" t="s">
         <v>55</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>79</v>
@@ -7929,12 +7939,12 @@
         <v>79</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="7" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B40" s="7" t="s">
         <v>55</v>
@@ -7943,7 +7953,7 @@
         <v>2</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="E40" s="7" t="s">
         <v>79</v>
@@ -7952,12 +7962,12 @@
         <v>79</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A41" s="7" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B41" s="7" t="s">
         <v>76</v>
@@ -7966,7 +7976,7 @@
         <v>2</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="E41" s="7" t="s">
         <v>79</v>
@@ -7975,64 +7985,64 @@
         <v>79</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
+        <v>480</v>
+      </c>
+      <c r="B42" t="s">
+        <v>55</v>
+      </c>
+      <c r="C42" t="s">
+        <v>405</v>
+      </c>
+      <c r="D42" t="s">
+        <v>481</v>
+      </c>
+      <c r="E42" t="s">
         <v>482</v>
       </c>
-      <c r="B42" t="s">
-        <v>55</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="F42" t="s">
         <v>407</v>
       </c>
-      <c r="D42" t="s">
+      <c r="G42" t="s">
         <v>483</v>
       </c>
-      <c r="E42" t="s">
-        <v>484</v>
-      </c>
-      <c r="F42" t="s">
-        <v>409</v>
-      </c>
-      <c r="G42" t="s">
-        <v>485</v>
-      </c>
     </row>
     <row r="43" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="32" t="s">
+      <c r="A43" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="B43" s="33"/>
-      <c r="C43" s="33"/>
-      <c r="D43" s="33"/>
-      <c r="E43" s="33"/>
-      <c r="F43" s="33"/>
-      <c r="G43" s="34"/>
+      <c r="B43" s="43"/>
+      <c r="C43" s="43"/>
+      <c r="D43" s="43"/>
+      <c r="E43" s="43"/>
+      <c r="F43" s="43"/>
+      <c r="G43" s="44"/>
     </row>
     <row r="44" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="35" t="s">
+      <c r="A44" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="B44" s="36"/>
-      <c r="C44" s="36"/>
-      <c r="D44" s="36"/>
-      <c r="E44" s="36"/>
-      <c r="F44" s="36"/>
-      <c r="G44" s="37"/>
+      <c r="B44" s="46"/>
+      <c r="C44" s="46"/>
+      <c r="D44" s="46"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="47"/>
     </row>
     <row r="45" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A45" s="38" t="s">
+      <c r="A45" s="48" t="s">
         <v>158</v>
       </c>
-      <c r="B45" s="39"/>
-      <c r="C45" s="39"/>
-      <c r="D45" s="39"/>
-      <c r="E45" s="39"/>
-      <c r="F45" s="39"/>
-      <c r="G45" s="40"/>
+      <c r="B45" s="49"/>
+      <c r="C45" s="49"/>
+      <c r="D45" s="49"/>
+      <c r="E45" s="49"/>
+      <c r="F45" s="49"/>
+      <c r="G45" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
[auto] session sync 2026-07-24T03:23:43Z
</commit_message>
<xml_diff>
--- a/2D 자동 제작도 개발 현황.xlsx
+++ b/2D 자동 제작도 개발 현황.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현황 요약" sheetId="1" r:id="Re18135f7cc0d4a33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개발 항목" sheetId="2" r:id="R90f8d174701f49ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항·UDA" sheetId="3" r:id="R6df1991648154a3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현황 요약" sheetId="1" r:id="R9eed27be84864170"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개발 항목" sheetId="2" r:id="R6b4d149df13a4f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항·UDA" sheetId="3" r:id="R0727e455856b4208"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1027,7 +1027,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="표준" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="50">
+  <x:dxfs count="56">
     <x:dxf/>
     <x:dxf/>
     <x:dxf/>
@@ -1378,6 +1378,72 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C6500"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1F4E78"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDEBF7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF8CBAD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF222222"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7E6E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
@@ -1995,7 +2061,7 @@
         <x:v>제작·가공·설치도 최종 PDF와 설명 장표</x:v>
       </x:c>
       <x:c r="D17" s="8" t="str">
-        <x:v>개발 중</x:v>
+        <x:v>개발 대기</x:v>
       </x:c>
       <x:c r="E17" s="7" t="str">
         <x:v>과제 완료 기준</x:v>
@@ -6046,7 +6112,7 @@
         <x:v>X</x:v>
       </x:c>
       <x:c r="I77" s="50" t="str">
-        <x:v>개발 중</x:v>
+        <x:v>개발 대기</x:v>
       </x:c>
       <x:c r="J77" s="51" t="str">
         <x:v>제작도·가공도·설치도 최종 PDF와 메뉴얼·룰북 설명 장표 필요</x:v>
@@ -6097,7 +6163,7 @@
         <x:v>해당없음</x:v>
       </x:c>
       <x:c r="I78" s="50" t="str">
-        <x:v>개발 중</x:v>
+        <x:v>개발 대기</x:v>
       </x:c>
       <x:c r="J78" s="51" t="str">
         <x:v>왼쪽 탭·테이블과 STRU 검색 상자의 배치·가독성 개선 필요</x:v>
@@ -6817,22 +6883,22 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="I6:I90">
-    <x:cfRule type="expression" dxfId="44" priority="28">
+    <x:cfRule type="expression" dxfId="50" priority="28">
       <x:formula>$I6="완료"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="45" priority="29">
+    <x:cfRule type="expression" dxfId="51" priority="29">
       <x:formula>$I6="실기 검증 대기"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="46" priority="30">
+    <x:cfRule type="expression" dxfId="52" priority="30">
       <x:formula>OR($I6="부분 구현",$I6="개발 중")</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="47" priority="31">
+    <x:cfRule type="expression" dxfId="53" priority="31">
       <x:formula>OR($I6="개발 필요",$I6="개발 대기")</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="48" priority="32">
+    <x:cfRule type="expression" dxfId="54" priority="32">
       <x:formula>OR($I6="분석 필요",$I6="적용 제외")</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="49" priority="33">
+    <x:cfRule type="expression" dxfId="55" priority="33">
       <x:formula>OR($I6="출력 불가",$I6="API 요청 필요",$I6="API 대기")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -6861,7 +6927,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2729326ffcea4f3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39b817ca4fc743f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>